<commit_message>
Scope socket.io to converter pages, shrink og-image, Western demo sample
og-image: 1.45 MB -> 40 KB, redrawn in the ledger system. socket.io
loads only on the dashboard (processing polls via fetch). Demo sample
regenerated with neutral Western transactions and reconverted through
the real parser.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/static/sample-statement.xlsx
+++ b/static/sample-statement.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="sheet1" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Full_Text" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Full_Text" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'sheet1'!$A$1:$E$7</definedName>
@@ -435,42 +435,42 @@
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
     <col width="42" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>DATE</t>
+          <t>Date</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>DESCRIPTION</t>
+          <t>Description</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>DEBIT</t>
+          <t>Withdrawals</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>CREDIT</t>
+          <t>Deposits</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>BALANCE</t>
+          <t>Balance</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>01/06/2026</t>
+          <t>06/01/2026</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
@@ -489,12 +489,12 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>03/06/2026</t>
+          <t>06/03/2026</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>UPI-GROCERY MART</t>
+          <t>CARD PURCHASE - GROCERY</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
@@ -512,30 +512,30 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>07/06/2026</t>
+          <t>06/07/2026</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>SALARY CREDIT JUNE</t>
+          <t>DIRECT DEPOSIT - EMPLOYER</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr"/>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>55,000.00</t>
+          <t>5,500.00</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>67,050.00</t>
+          <t>17,550.00</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>12/06/2026</t>
+          <t>06/12/2026</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
@@ -545,59 +545,59 @@
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>5,000.00</t>
+          <t>500.00</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr"/>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>62,050.00</t>
+          <t>17,050.00</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>18/06/2026</t>
+          <t>06/18/2026</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>ELECTRICITY BILL</t>
+          <t>ACH PAYMENT - UTILITIES</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>1,240.00</t>
+          <t>124.00</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr"/>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>60,810.00</t>
+          <t>16,926.00</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>25/06/2026</t>
+          <t>06/25/2026</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>FD INTEREST</t>
+          <t>INTEREST PAYMENT</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr"/>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>820.00</t>
+          <t>8.20</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>61,630.00</t>
+          <t>16,934.20</t>
         </is>
       </c>
     </row>
@@ -613,7 +613,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D9"/>
+  <dimension ref="A1:D10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -662,7 +662,7 @@
       </c>
       <c r="D2" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">        DEMO BANK - Account Statement 01/06/2026 to 30/06/2026</t>
+          <t xml:space="preserve">      DEMO BANK</t>
         </is>
       </c>
     </row>
@@ -684,7 +684,7 @@
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">         DATE        DESCRIPTION                DEBIT         CREDIT        BALANCE</t>
+          <t xml:space="preserve">        Account Statement 06/01/2026 - 06/30/2026</t>
         </is>
       </c>
     </row>
@@ -706,7 +706,7 @@
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">          01/06/2026     OPENING BALANCE                12,500.00</t>
+          <t xml:space="preserve">          Date          Description                Withdrawals        Deposits         Balance</t>
         </is>
       </c>
     </row>
@@ -728,7 +728,7 @@
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">           03/06/2026     UPI-GROCERY MART                450.00                12,050.00</t>
+          <t xml:space="preserve">          06/01/2026     OPENING BALANCE                12,500.00</t>
         </is>
       </c>
     </row>
@@ -750,7 +750,7 @@
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">          07/06/2026     SALARY CREDIT JUNE                55,000.00        67,050.00</t>
+          <t xml:space="preserve">           06/03/2026     CARD PURCHASE - GROCERY                450.00                12,050.00</t>
         </is>
       </c>
     </row>
@@ -772,7 +772,7 @@
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">           12/06/2026      ATM WITHDRAWAL                5,000.00                62,050.00</t>
+          <t xml:space="preserve">           06/07/2026      DIRECT DEPOSIT - EMPLOYER                5,500.00          17,550.00</t>
         </is>
       </c>
     </row>
@@ -794,7 +794,7 @@
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">           18/06/2026      ELECTRICITY BILL                1,240.00                60,810.00</t>
+          <t xml:space="preserve">           06/12/2026     ATM WITHDRAWAL                500.00                17,050.00</t>
         </is>
       </c>
     </row>
@@ -816,7 +816,29 @@
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">           25/06/2026     FD INTEREST                820.00           61,630.00</t>
+          <t xml:space="preserve">           06/18/2026     ACH PAYMENT - UTILITIES                124.00                16,926.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>pdf-text</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">           06/25/2026      INTEREST PAYMENT                8.20              16,934.20</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Improve layout fidelity and OCR verification
</commit_message>
<xml_diff>
--- a/static/sample-statement.xlsx
+++ b/static/sample-statement.xlsx
@@ -7,11 +7,12 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="sheet1" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Full_Text" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Exact_Copy" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table_Data" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Full_Text" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'sheet1'!$A$1:$E$7</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Table_Data'!$A$1:$E$7</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -61,9 +62,11 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="49" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -430,6 +433,386 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:CF10"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="1.6" customWidth="1" min="1" max="1"/>
+    <col width="1.6" customWidth="1" min="2" max="2"/>
+    <col width="1.6" customWidth="1" min="3" max="3"/>
+    <col width="1.6" customWidth="1" min="4" max="4"/>
+    <col width="1.6" customWidth="1" min="5" max="5"/>
+    <col width="1.6" customWidth="1" min="6" max="6"/>
+    <col width="1.6" customWidth="1" min="7" max="7"/>
+    <col width="1.6" customWidth="1" min="8" max="8"/>
+    <col width="1.6" customWidth="1" min="9" max="9"/>
+    <col width="1.6" customWidth="1" min="10" max="10"/>
+    <col width="1.6" customWidth="1" min="11" max="11"/>
+    <col width="1.6" customWidth="1" min="12" max="12"/>
+    <col width="1.6" customWidth="1" min="13" max="13"/>
+    <col width="1.6" customWidth="1" min="14" max="14"/>
+    <col width="1.6" customWidth="1" min="15" max="15"/>
+    <col width="1.6" customWidth="1" min="16" max="16"/>
+    <col width="1.6" customWidth="1" min="17" max="17"/>
+    <col width="1.6" customWidth="1" min="18" max="18"/>
+    <col width="1.6" customWidth="1" min="19" max="19"/>
+    <col width="1.6" customWidth="1" min="20" max="20"/>
+    <col width="1.6" customWidth="1" min="21" max="21"/>
+    <col width="1.6" customWidth="1" min="22" max="22"/>
+    <col width="1.6" customWidth="1" min="23" max="23"/>
+    <col width="1.6" customWidth="1" min="24" max="24"/>
+    <col width="1.6" customWidth="1" min="25" max="25"/>
+    <col width="1.6" customWidth="1" min="26" max="26"/>
+    <col width="1.6" customWidth="1" min="27" max="27"/>
+    <col width="1.6" customWidth="1" min="28" max="28"/>
+    <col width="1.6" customWidth="1" min="29" max="29"/>
+    <col width="1.6" customWidth="1" min="30" max="30"/>
+    <col width="1.6" customWidth="1" min="31" max="31"/>
+    <col width="1.6" customWidth="1" min="32" max="32"/>
+    <col width="1.6" customWidth="1" min="33" max="33"/>
+    <col width="1.6" customWidth="1" min="34" max="34"/>
+    <col width="1.6" customWidth="1" min="35" max="35"/>
+    <col width="1.6" customWidth="1" min="36" max="36"/>
+    <col width="1.6" customWidth="1" min="37" max="37"/>
+    <col width="1.6" customWidth="1" min="38" max="38"/>
+    <col width="1.6" customWidth="1" min="39" max="39"/>
+    <col width="1.6" customWidth="1" min="40" max="40"/>
+    <col width="1.6" customWidth="1" min="41" max="41"/>
+    <col width="1.6" customWidth="1" min="42" max="42"/>
+    <col width="1.6" customWidth="1" min="43" max="43"/>
+    <col width="1.6" customWidth="1" min="44" max="44"/>
+    <col width="1.6" customWidth="1" min="45" max="45"/>
+    <col width="1.6" customWidth="1" min="46" max="46"/>
+    <col width="1.6" customWidth="1" min="47" max="47"/>
+    <col width="1.6" customWidth="1" min="48" max="48"/>
+    <col width="1.6" customWidth="1" min="49" max="49"/>
+    <col width="1.6" customWidth="1" min="50" max="50"/>
+    <col width="1.6" customWidth="1" min="51" max="51"/>
+    <col width="1.6" customWidth="1" min="52" max="52"/>
+    <col width="1.6" customWidth="1" min="53" max="53"/>
+    <col width="1.6" customWidth="1" min="54" max="54"/>
+    <col width="1.6" customWidth="1" min="55" max="55"/>
+    <col width="1.6" customWidth="1" min="56" max="56"/>
+    <col width="1.6" customWidth="1" min="57" max="57"/>
+    <col width="1.6" customWidth="1" min="58" max="58"/>
+    <col width="1.6" customWidth="1" min="59" max="59"/>
+    <col width="1.6" customWidth="1" min="60" max="60"/>
+    <col width="1.6" customWidth="1" min="61" max="61"/>
+    <col width="1.6" customWidth="1" min="62" max="62"/>
+    <col width="1.6" customWidth="1" min="63" max="63"/>
+    <col width="1.6" customWidth="1" min="64" max="64"/>
+    <col width="1.6" customWidth="1" min="65" max="65"/>
+    <col width="1.6" customWidth="1" min="66" max="66"/>
+    <col width="1.6" customWidth="1" min="67" max="67"/>
+    <col width="1.6" customWidth="1" min="68" max="68"/>
+    <col width="1.6" customWidth="1" min="69" max="69"/>
+    <col width="1.6" customWidth="1" min="70" max="70"/>
+    <col width="1.6" customWidth="1" min="71" max="71"/>
+    <col width="1.6" customWidth="1" min="72" max="72"/>
+    <col width="1.6" customWidth="1" min="73" max="73"/>
+    <col width="1.6" customWidth="1" min="74" max="74"/>
+    <col width="1.6" customWidth="1" min="75" max="75"/>
+    <col width="1.6" customWidth="1" min="76" max="76"/>
+    <col width="1.6" customWidth="1" min="77" max="77"/>
+    <col width="1.6" customWidth="1" min="78" max="78"/>
+    <col width="1.6" customWidth="1" min="79" max="79"/>
+    <col width="1.6" customWidth="1" min="80" max="80"/>
+    <col width="1.6" customWidth="1" min="81" max="81"/>
+    <col width="1.6" customWidth="1" min="82" max="82"/>
+    <col width="1.6" customWidth="1" min="83" max="83"/>
+    <col width="1.6" customWidth="1" min="84" max="84"/>
+    <col width="1.6" customWidth="1" min="85" max="85"/>
+    <col width="1.6" customWidth="1" min="86" max="86"/>
+    <col width="1.6" customWidth="1" min="87" max="87"/>
+    <col width="1.6" customWidth="1" min="88" max="88"/>
+    <col width="1.6" customWidth="1" min="89" max="89"/>
+    <col width="1.6" customWidth="1" min="90" max="90"/>
+    <col width="1.6" customWidth="1" min="91" max="91"/>
+    <col width="1.6" customWidth="1" min="92" max="92"/>
+    <col width="1.6" customWidth="1" min="93" max="93"/>
+    <col width="1.6" customWidth="1" min="94" max="94"/>
+    <col width="1.6" customWidth="1" min="95" max="95"/>
+    <col width="1.6" customWidth="1" min="96" max="96"/>
+    <col width="1.6" customWidth="1" min="97" max="97"/>
+    <col width="1.6" customWidth="1" min="98" max="98"/>
+    <col width="1.6" customWidth="1" min="99" max="99"/>
+    <col width="1.6" customWidth="1" min="100" max="100"/>
+    <col width="1.6" customWidth="1" min="101" max="101"/>
+    <col width="1.6" customWidth="1" min="102" max="102"/>
+    <col width="1.6" customWidth="1" min="103" max="103"/>
+    <col width="1.6" customWidth="1" min="104" max="104"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Page 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="15" customHeight="1">
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>DEMO</t>
+        </is>
+      </c>
+      <c r="P2" s="2" t="inlineStr">
+        <is>
+          <t>BANK</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="15" customHeight="1">
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>Account</t>
+        </is>
+      </c>
+      <c r="R3" s="2" t="inlineStr">
+        <is>
+          <t>Statement</t>
+        </is>
+      </c>
+      <c r="AB3" s="2" t="inlineStr">
+        <is>
+          <t>06/01/2026</t>
+        </is>
+      </c>
+      <c r="AM3" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AN3" s="2" t="inlineStr">
+        <is>
+          <t>06/30/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="12" customHeight="1">
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="U4" s="2" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="BD4" s="2" t="inlineStr">
+        <is>
+          <t>Withdrawals</t>
+        </is>
+      </c>
+      <c r="BS4" s="2" t="inlineStr">
+        <is>
+          <t>Deposits</t>
+        </is>
+      </c>
+      <c r="CF4" s="2" t="inlineStr">
+        <is>
+          <t>Balance</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="12" customHeight="1">
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>06/01/2026</t>
+        </is>
+      </c>
+      <c r="U5" s="2" t="inlineStr">
+        <is>
+          <t>OPENING</t>
+        </is>
+      </c>
+      <c r="AB5" s="2" t="inlineStr">
+        <is>
+          <t>BALANCE</t>
+        </is>
+      </c>
+      <c r="CF5" s="2" t="inlineStr">
+        <is>
+          <t>12,500.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="12" customHeight="1">
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>06/03/2026</t>
+        </is>
+      </c>
+      <c r="U6" s="2" t="inlineStr">
+        <is>
+          <t>CARD</t>
+        </is>
+      </c>
+      <c r="Z6" s="2" t="inlineStr">
+        <is>
+          <t>PURCHASE</t>
+        </is>
+      </c>
+      <c r="AH6" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AI6" s="2" t="inlineStr">
+        <is>
+          <t>GROCERY</t>
+        </is>
+      </c>
+      <c r="BD6" s="2" t="inlineStr">
+        <is>
+          <t>450.00</t>
+        </is>
+      </c>
+      <c r="CF6" s="2" t="inlineStr">
+        <is>
+          <t>12,050.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="12" customHeight="1">
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>06/07/2026</t>
+        </is>
+      </c>
+      <c r="U7" s="2" t="inlineStr">
+        <is>
+          <t>DIRECT</t>
+        </is>
+      </c>
+      <c r="AA7" s="2" t="inlineStr">
+        <is>
+          <t>DEPOSIT</t>
+        </is>
+      </c>
+      <c r="AH7" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AI7" s="2" t="inlineStr">
+        <is>
+          <t>EMPLOYER</t>
+        </is>
+      </c>
+      <c r="BS7" s="2" t="inlineStr">
+        <is>
+          <t>5,500.00</t>
+        </is>
+      </c>
+      <c r="CF7" s="2" t="inlineStr">
+        <is>
+          <t>17,550.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="12" customHeight="1">
+      <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t>06/12/2026</t>
+        </is>
+      </c>
+      <c r="U8" s="2" t="inlineStr">
+        <is>
+          <t>ATM</t>
+        </is>
+      </c>
+      <c r="Y8" s="2" t="inlineStr">
+        <is>
+          <t>WITHDRAWAL</t>
+        </is>
+      </c>
+      <c r="BD8" s="2" t="inlineStr">
+        <is>
+          <t>500.00</t>
+        </is>
+      </c>
+      <c r="CF8" s="2" t="inlineStr">
+        <is>
+          <t>17,050.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="12" customHeight="1">
+      <c r="I9" s="2" t="inlineStr">
+        <is>
+          <t>06/18/2026</t>
+        </is>
+      </c>
+      <c r="U9" s="2" t="inlineStr">
+        <is>
+          <t>ACH</t>
+        </is>
+      </c>
+      <c r="Y9" s="2" t="inlineStr">
+        <is>
+          <t>PAYMENT</t>
+        </is>
+      </c>
+      <c r="AF9" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AG9" s="2" t="inlineStr">
+        <is>
+          <t>UTILITIES</t>
+        </is>
+      </c>
+      <c r="BD9" s="2" t="inlineStr">
+        <is>
+          <t>124.00</t>
+        </is>
+      </c>
+      <c r="CF9" s="2" t="inlineStr">
+        <is>
+          <t>16,926.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="12" customHeight="1">
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t>06/25/2026</t>
+        </is>
+      </c>
+      <c r="U10" s="2" t="inlineStr">
+        <is>
+          <t>INTEREST</t>
+        </is>
+      </c>
+      <c r="AC10" s="2" t="inlineStr">
+        <is>
+          <t>PAYMENT</t>
+        </is>
+      </c>
+      <c r="BS10" s="2" t="inlineStr">
+        <is>
+          <t>8.20</t>
+        </is>
+      </c>
+      <c r="CF10" s="2" t="inlineStr">
+        <is>
+          <t>16,934.20</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:E7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -468,134 +851,134 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" s="3" t="inlineStr">
         <is>
           <t>06/01/2026</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr">
+      <c r="B2" s="3" t="inlineStr">
         <is>
           <t>OPENING BALANCE</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr"/>
-      <c r="D2" s="2" t="inlineStr"/>
-      <c r="E2" s="2" t="inlineStr">
+      <c r="C2" s="3" t="inlineStr"/>
+      <c r="D2" s="3" t="inlineStr"/>
+      <c r="E2" s="3" t="inlineStr">
         <is>
           <t>12,500.00</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
+      <c r="A3" s="3" t="inlineStr">
         <is>
           <t>06/03/2026</t>
         </is>
       </c>
-      <c r="B3" s="2" t="inlineStr">
+      <c r="B3" s="3" t="inlineStr">
         <is>
           <t>CARD PURCHASE - GROCERY</t>
         </is>
       </c>
-      <c r="C3" s="2" t="inlineStr">
+      <c r="C3" s="3" t="inlineStr">
         <is>
           <t>450.00</t>
         </is>
       </c>
-      <c r="D3" s="2" t="inlineStr"/>
-      <c r="E3" s="2" t="inlineStr">
+      <c r="D3" s="3" t="inlineStr"/>
+      <c r="E3" s="3" t="inlineStr">
         <is>
           <t>12,050.00</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="inlineStr">
+      <c r="A4" s="3" t="inlineStr">
         <is>
           <t>06/07/2026</t>
         </is>
       </c>
-      <c r="B4" s="2" t="inlineStr">
+      <c r="B4" s="3" t="inlineStr">
         <is>
           <t>DIRECT DEPOSIT - EMPLOYER</t>
         </is>
       </c>
-      <c r="C4" s="2" t="inlineStr"/>
-      <c r="D4" s="2" t="inlineStr">
+      <c r="C4" s="3" t="inlineStr"/>
+      <c r="D4" s="3" t="inlineStr">
         <is>
           <t>5,500.00</t>
         </is>
       </c>
-      <c r="E4" s="2" t="inlineStr">
+      <c r="E4" s="3" t="inlineStr">
         <is>
           <t>17,550.00</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="inlineStr">
+      <c r="A5" s="3" t="inlineStr">
         <is>
           <t>06/12/2026</t>
         </is>
       </c>
-      <c r="B5" s="2" t="inlineStr">
+      <c r="B5" s="3" t="inlineStr">
         <is>
           <t>ATM WITHDRAWAL</t>
         </is>
       </c>
-      <c r="C5" s="2" t="inlineStr">
+      <c r="C5" s="3" t="inlineStr">
         <is>
           <t>500.00</t>
         </is>
       </c>
-      <c r="D5" s="2" t="inlineStr"/>
-      <c r="E5" s="2" t="inlineStr">
+      <c r="D5" s="3" t="inlineStr"/>
+      <c r="E5" s="3" t="inlineStr">
         <is>
           <t>17,050.00</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="inlineStr">
+      <c r="A6" s="3" t="inlineStr">
         <is>
           <t>06/18/2026</t>
         </is>
       </c>
-      <c r="B6" s="2" t="inlineStr">
+      <c r="B6" s="3" t="inlineStr">
         <is>
           <t>ACH PAYMENT - UTILITIES</t>
         </is>
       </c>
-      <c r="C6" s="2" t="inlineStr">
+      <c r="C6" s="3" t="inlineStr">
         <is>
           <t>124.00</t>
         </is>
       </c>
-      <c r="D6" s="2" t="inlineStr"/>
-      <c r="E6" s="2" t="inlineStr">
+      <c r="D6" s="3" t="inlineStr"/>
+      <c r="E6" s="3" t="inlineStr">
         <is>
           <t>16,926.00</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="inlineStr">
+      <c r="A7" s="3" t="inlineStr">
         <is>
           <t>06/25/2026</t>
         </is>
       </c>
-      <c r="B7" s="2" t="inlineStr">
+      <c r="B7" s="3" t="inlineStr">
         <is>
           <t>INTEREST PAYMENT</t>
         </is>
       </c>
-      <c r="C7" s="2" t="inlineStr"/>
-      <c r="D7" s="2" t="inlineStr">
+      <c r="C7" s="3" t="inlineStr"/>
+      <c r="D7" s="3" t="inlineStr">
         <is>
           <t>8.20</t>
         </is>
       </c>
-      <c r="E7" s="2" t="inlineStr">
+      <c r="E7" s="3" t="inlineStr">
         <is>
           <t>16,934.20</t>
         </is>
@@ -607,7 +990,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -623,22 +1006,22 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="3" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Page</t>
         </is>
       </c>
-      <c r="B1" s="3" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Line</t>
         </is>
       </c>
-      <c r="C1" s="3" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Source</t>
         </is>
       </c>
-      <c r="D1" s="3" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Text</t>
         </is>

</xml_diff>